<commit_message>
feat: Add Explorer, Hero, Innocent, Jester, Lover, Magician, Outlaw pour batches, reworks, and enriched archetype narratives
</commit_message>
<xml_diff>
--- a/Cocktail_GPT/Brand Personality + Roulette.xlsx
+++ b/Cocktail_GPT/Brand Personality + Roulette.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1902" uniqueCount="983">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1902" uniqueCount="1160">
   <si>
     <t>ARCHETYPE</t>
   </si>
@@ -3187,6 +3187,559 @@
   </si>
   <si>
     <t>Observing the world form the outside, living outside of society, and being unaware of the convention of it.</t>
+  </si>
+  <si>
+    <t>Taking care of the things that you uncover and seeking to understand the world better for the good of humankind</t>
+  </si>
+  <si>
+    <t>Sir David Attenborough</t>
+  </si>
+  <si>
+    <t>Like David Attenborough, who has spent more than seventy years getting close to wild things without ever wanting to own them, the Conservationist goes out into the world to see it as it really is. Their freedom comes with a duty attached: whatever they find, they feel responsible for. They travel light, leave no trace and notice what is disappearing before anyone else does. What haunts them is coming back one day to find that the place they loved is gone.</t>
+  </si>
+  <si>
+    <t>The Innovator cannot stand living inside an answer someone else settled on. James Dyson got so fed up with a vacuum cleaner that kept losing its suction that it took five years and thousands of prototypes to build a way out. That is their pattern: irritation first, then the workshop, then a door nobody knew was there. They invent to escape, and every new thing they make is a little more room to breathe. Being handed a finished world and told to live in it is their idea of a cage.</t>
+  </si>
+  <si>
+    <t>The Tourist wants the world, with a return ticket in their pocket. They follow the guidebook, then take one street further, into the café with no menu in their language, and come home glowing about it. They don't want to vanish into a place. They want to share it: the photos, the tips, the story told over dinner. Adventure feels best to them with company and a way back. Being stuck, even somewhere beautiful, is the one trip they would never book.</t>
+  </si>
+  <si>
+    <t>The Pioneer goes where no one has been, knowing everyone is watching. Neil Armstrong trained for years for a few hours on the Moon, stayed calm through a landing that nearly ran out of fuel, and called it one small step. Pioneers carry their fear quietly, because the moment needs a steady pair of hands. The new ground is their freedom and their proof. What they could never live with is having been ready, and not gone.</t>
+  </si>
+  <si>
+    <t>The Discoverer never quite stopped asking why. Late in life, Newton told a friend that the idea of gravity first came to him while watching an apple fall in his mother's garden, a thing millions had seen and nobody had wondered about. That is their gift: they stay open long enough for the ordinary to turn strange. They trust the world to be interesting, and it usually obliges. A life too busy and too certain to be surprised by anything is the trap they keep stepping around.</t>
+  </si>
+  <si>
+    <t>Wallace &amp; Gromit</t>
+  </si>
+  <si>
+    <t>The Mad Inventor would rather build a machine to make breakfast than simply make breakfast. Like Wallace down in the cellar in Wallace &amp; Gromit, they tinker for the joy of it. Rules are closed doors, and they like every door open. Half their ideas collapse in a heap of springs, and they laugh the loudest. The other half work, to everyone's surprise, including their own. Nothing deflates them faster than being told to be sensible.</t>
+  </si>
+  <si>
+    <t>Exploring the senses, seeking stimulation and discovering new sensory experiences</t>
+  </si>
+  <si>
+    <t>The Sense Seeker travels by taste, by smell, by fingertip. Like Nigel Slater, who told the story of his own childhood through the food he ate, they remember a city by its bakeries and a summer by one perfect peach. Adventure, for them, is close up: an unfamiliar spice, a stranger's kitchen, the market before it opens. They want an appetite that nobody has to approve. The life they dread is a grey one, where every day tastes the same.</t>
+  </si>
+  <si>
+    <t>The Spiritualist travels in two directions at once: outward, to monasteries, retreats and long walks, and inward, towards whatever is quiet under the noise. They read everything from ancient scripture to The Secret and keep the one line that changes them. They believe a mind can be transformed, and that happiness is something to go out and find rather than wait for. What frightens them is an ordinary life that never once asks what it is for.</t>
+  </si>
+  <si>
+    <t>The Trailblazer doesn't wait for a path to be approved. Edmund Hillary was a beekeeper from New Zealand when he joined the 1953 British expedition to Everest, and he came down from the summit telling a friend, 'We knocked the bastard off.' That mix of nerve and irreverence is the Trailblazer all over. Rules are for people who want to be told where to go. The fenced field and the signposted route are their idea of a prison.</t>
+  </si>
+  <si>
+    <t>The Expedition Leader</t>
+  </si>
+  <si>
+    <t>Ernest Shackleton</t>
+  </si>
+  <si>
+    <t>The Expedition Leader goes into the unknown with other people's lives in their hands, and brings everyone home. When Antarctic ice trapped and crushed Shackleton's ship Endurance, he kept the crew hopeful for well over a year, then crossed 800 miles of the Southern Ocean in an open boat to fetch help. Not one of the crew died. This person loves the wild edge of the map and the discipline it takes to survive there. Being trapped is their worst fear, and when it happens anyway, they don't panic. They organise.</t>
+  </si>
+  <si>
+    <t>For the Genius, the mind is the one place nobody can fence in. Einstein hated the drill of his school days, and at sixteen was already imagining what it would be like to chase a beam of light. The papers that changed physics came from a patent clerk in Bern. That is how they explore: one question held loosely for years, until it turns the world over. They trust evidence and distrust any authority that can't explain itself. A desk where thinking isn't allowed would suffocate them.</t>
+  </si>
+  <si>
+    <t>The Saviour</t>
+  </si>
+  <si>
+    <t>Completely selfless and would give themselves up to benefit others</t>
+  </si>
+  <si>
+    <t>The Saviour is the one who steps forward when everyone else steps back, ready to give up their own comfort, or far more, so that someone else is spared. The story of Jesus made that kind of love the most familiar in the world. What people rarely see is the other side: the Saviour finds it very hard to be saved. Needing help feels like weakness to them, so they carry more than anyone should and call it duty.</t>
+  </si>
+  <si>
+    <t>The Idealist fights with songs, words and pictures instead of fists. In the early sixties Bob Dylan wrote lines that civil rights marchers sang in the streets, and then, crowned the voice of a generation, refused the crown and kept changing. That is the Idealist: brave enough to stand for something, stubborn enough not to become anyone's slogan. They want the world a little fairer when they leave it. Going quiet when it matters is the failure they fear most.</t>
+  </si>
+  <si>
+    <t>The Firefighter</t>
+  </si>
+  <si>
+    <t>Anyone would have done the same; the everyday hero.</t>
+  </si>
+  <si>
+    <t>9/11 firefighters</t>
+  </si>
+  <si>
+    <t>The Firefighter runs towards what everyone else runs from, then shrugs it off: anyone would have done the same. Not everyone would, and they know it, which is why they train so hard for the few minutes that count. On 11 September 2001, New York's firefighters climbed the stairs of the burning towers as thousands came down. This person's courage is practised, shared with a crew and never shown off. Deep down, they are afraid of not being good enough on the day someone needs them.</t>
+  </si>
+  <si>
+    <t>Travels to the end of the world to find the reward and bring it back. Never held back by fear, always courageous and daring</t>
+  </si>
+  <si>
+    <t>The Quest Seeker needs something to go after: a lost object, a hard answer, a summit with a name. Indiana Jones crosses deserts and collapsing temples for a relic and is terrified of snakes the whole way. That is the truth of this person. The fear comes along, and they go anyway. The prize matters, but what they really bring home is proof that they could. A life with nothing left to find scares them more than any snake.</t>
+  </si>
+  <si>
+    <t>Facing challenges for the first time with the bravery, optimism and vitality of youth. They must face and overcome their challenges to become a true hero.</t>
+  </si>
+  <si>
+    <t>The Initiate is at the very start of becoming someone. Like Luke Skywalker watching two suns set over a farm at the edge of nowhere, they feel certain there is more to them than this, without a shred of proof yet. They are brave the way beginners are brave, unsure and willing, and every trial they survive makes them a little more themselves. They trust their mentors, sometimes too quickly. The moment they dread is the one where it counts, and they turn out not to be ready.</t>
+  </si>
+  <si>
+    <t>The Storyteller</t>
+  </si>
+  <si>
+    <t>The Storyteller can turn a flat tyre into an epic. Like Edward Bloom in Big Fish, whose tall tales of giants and witches drive a truth-hungry son to despair, they make life larger in the telling, and everyone leans in. People take them for show-offs. The truth is kinder. They tell their struggles as adventures so the struggle doesn't win, and so that others believe they can come through theirs. What frightens them is a plain life, told plainly, that nobody remembers.</t>
+  </si>
+  <si>
+    <t>Swashbuckling, heroic and always lands on their feet</t>
+  </si>
+  <si>
+    <t>The Dashing Hero makes danger look like a dance: calm under fire, a joke ready, a perfectly timed exit. James Bond is the famous version, all nerve and polish. But the Dashing Hero is never brave for nothing. Underneath the style is someone who fights for the people they love and hides how much they love them, because feeling too much looks like weakness. Losing someone they could not protect is the wound they never show.</t>
+  </si>
+  <si>
+    <t>The Superhero lives a double life. Like Clark Kent, they can seem ordinary, even a little awkward, while carrying abilities that could change a room, a company or a life. Every day they choose to use that power for others, and to hold it back when it would only show off. The hardest part isn't the rescue. It is being loved for the cape rather than the person underneath, and the quiet fear that without the cape they would be nothing special.</t>
+  </si>
+  <si>
+    <t>Pirates of the Caribbean (Jack Sparrow), Luffy</t>
+  </si>
+  <si>
+    <t>The Lovable Rogue looks like the last person anyone would trust with something important, and turns out to be the one who comes back. Like Jack Sparrow, they bend every rule, make the plan up as they go and hide a real sense of honour behind a joke. They hate being told what to do, but they hate letting a friend down more. Being thought soft is their horror, so the kindness always arrives with a wink.</t>
+  </si>
+  <si>
+    <t>Troy (Hector)</t>
+  </si>
+  <si>
+    <t>The Warrior stands in front so that others can stand behind. In Troy it is Hector who carries the weight of the city: training, commanding and, at the end, walking out alone through the gates to face Achilles. This person trusts discipline more than luck and leads by being first into difficulty. They keep order when things fall apart because someone has to. What they fear is not the fight but faltering in front of the people who depend on them.</t>
+  </si>
+  <si>
+    <t>The Problem Solver gets calmer as things get worse. While others panic, they are already asking the useful questions: what do we know, what do we have, what happens if we try this? A riddle delights them, and a crisis is simply a riddle with a clock on it. It takes nerve to think clearly under pressure, and they have it. The nightmare is standing in front of a problem, with everyone watching, and having no answer.</t>
+  </si>
+  <si>
+    <t>The Big Sibling</t>
+  </si>
+  <si>
+    <t>The Big Sibling learned to look after someone before they learned to look after themselves. They were the child who held the smaller hand at the crossing, saved the last biscuit for someone else and stayed awake when the little one was scared of the dark. None of it was calculated. It simply seemed obvious that the people they love should be safe. Grown up, they still check that everyone got home. The fear that never left them is someone getting hurt on their watch.</t>
+  </si>
+  <si>
+    <t>Observing the world from the outside, living outside of society, and being unaware of its conventions.</t>
+  </si>
+  <si>
+    <t>The Naive Artist makes things the way children draw, before anyone has told them what is correct. They paint the sky the colour it felt, give a cat the dignity of a king and break rules without noticing, because nobody taught them the rules. Jean Dubuffet called this kind of work art brut, raw art, and prized it above polish. They make things to share a world that seems simply, obviously beautiful. What they fear is being laughed at, and then learning to be careful.</t>
+  </si>
+  <si>
+    <t>The True Friend is the one who shows up. Like Woody and Buzz in Toy Story, who begin as rivals and end up chasing a removal van across town to get each other home, they choose loyalty over pride, forgive quickly and never keep score. They believe the best of people, and people tend to rise to it. The world feels kinder with them in it. What they fear is being left out, and, worse, a friend feeling alone when they could have been there.</t>
+  </si>
+  <si>
+    <t>Alice in Wonderland (Tim Burton)</t>
+  </si>
+  <si>
+    <t>The Free Spirit follows the White Rabbit. Like Alice, they tumble into strange places and meet them with questions instead of fear: why is this door so small, and why must the Queen always be obeyed? They trust the world to be wonderful, and the trust makes them brave. Grown-up rules puzzle them more than they frighten them. What would break their heart is a world so explained and so labelled that nothing is left to wonder at.</t>
+  </si>
+  <si>
+    <t>The Underdog never set out to win anything. In Slumdog Millionaire, Jamal ends up one question from a fortune, not through cleverness or cunning, but because life has taught him every answer the hard way, and the only prize that matters is finding Latika. That is the Underdog: good without a strategy, brave without noticing. They are usually the last to realise how far they have come. Their fear is being accused of cheating when they have only ever played it straight.</t>
+  </si>
+  <si>
+    <t>The Giggler finds something funny in almost everything and can't keep it in. Like Mr Tickle stretching those extraordinarily long arms through windows and round corners, they reach into a serious room and set it laughing. Their mischief is never cruel. They simply can't believe everyone isn't enjoying this as much as they are. Laughter is how they know the world is safe. Being told off for it, and learning to be solemn, is what they dread.</t>
+  </si>
+  <si>
+    <t>The Teenage Heart-throb loves the way everyone did at fifteen: completely, out loud, with no plan for it ever ending. They write the note, make the playlist and say the big words first. It can look naive. It is actually brave, to care that much in public. Whole stadiums have sung that feeling back to Justin Bieber, because nobody forgets it. The day they dread is the one when someone calls it silly and they start loving more carefully.</t>
+  </si>
+  <si>
+    <t>The Dreamer believes that wishing, done properly, changes things. Like Dorothy in her ruby slippers, they follow the yellow brick road towards wonders and discover at the end that the magic was on their feet all along. They notice signs, trust their hunches and carry hope for people who have run out of it. Their quiet discovery is that there's no place like home, and that home is worth dreaming about too. Being scolded for hoping is what hurts them most.</t>
+  </si>
+  <si>
+    <t>The Outsider stepped out of the race, not to fight anyone but to stay clean of it. They would rather have a small life that is truly theirs than a big one built on other people's expectations. They trust nature, simple food, honest work and their own company. Into the Wild tells that longing, and what it can cost. The Outsider isn't angry. They simply refuse to be spoiled, and their fear is being pulled back in and made to compromise.</t>
+  </si>
+  <si>
+    <t>The Little Prince rules a very small world and takes it completely seriously. Every morning they pull up the baobab shoots before they can take over, and they tend one rose as if nothing else mattered, because to them nothing else does. Grown-ups' numbers and titles leave them puzzled. They see what matters with the heart, and they know, as the fox says, that 'you become responsible, forever, for what you have tamed.' Failing the one thing in their care is their deepest fear.</t>
+  </si>
+  <si>
+    <t>Sometimes the greatest wisdom comes from the mouths of the inexperienced. A naive observer who sees the truth of the matter.</t>
+  </si>
+  <si>
+    <t>The Wise Kid says the thing everyone else in the room is too clever to say. In About a Boy it is twelve-year-old Marcus, odd and unfashionable, who sees straight through Will's carefully idle cool and teaches him to care about someone. This person is often inexperienced and rarely wrong. They ask the simple question and wait for an honest answer. Being lied to by people they trust, or told that the truth is rude, is what wounds them.</t>
+  </si>
+  <si>
+    <t>A contagious and positive outlook on life that fills others with happiness. Makes us laugh, makes us feel better.</t>
+  </si>
+  <si>
+    <t>The Morale Booster walks into a heavy room and changes the weather. They know exactly when a joke will help and when it would hurt, and they use humour the way others use a blanket or a cup of tea. Hospital clowns do this for a living, making a frightened child laugh long enough to forget where they are. The fun this person makes is always for someone. What they can't bear is a gloom nobody can lift, and being the one who couldn't lift it.</t>
+  </si>
+  <si>
+    <t>The Wacky One turns the strange into a signature. They wear the odd hat, build the pointless machine and invent a word, then use it until everyone else does too. Like Popeye, all pipe, squint and spinach, they are ridiculous and completely at home in it: I yam what I yam. They make nonsense for the pleasure of it and for the freedom it gives everyone else. Being normal on purpose is the one thing they refuse to do.</t>
+  </si>
+  <si>
+    <t>The Stand-up notices what everyone does and nobody mentions: the pocket checked three times for keys, the friend who says 'five minutes' and means forty. Jerry Seinfeld built a whole show about nothing on exactly that, and it turned out to be about everyone. This person makes people feel normal by getting them to laugh at being human together. They are at their best at the table, not at the head of it. A dull evening where nobody says what they're thinking is their idea of torture.</t>
+  </si>
+  <si>
+    <t>Andy Kaufman</t>
+  </si>
+  <si>
+    <t>The Alternative Comic can't tell the same joke twice. Andy Kaufman once read The Great Gatsby aloud to an audience that had come for laughs, just to see what would happen when the laughter had nowhere to go. This person experiments with fun, pushing it somewhere new and slightly uncomfortable, where the joke is on the format itself. They would rather puzzle a crowd than please it the easy way. The familiar punchline bores them to tears.</t>
+  </si>
+  <si>
+    <t>Roberto Benigni in La vita è bella</t>
+  </si>
+  <si>
+    <t>The Wise Talker is still joking when everyone else has given up, and the joke is how they keep people going. In Life Is Beautiful, Roberto Benigni's Guido turns the horror of a concentration camp into a game, so that a small boy never loses hope. That is this person at their most heroic: humour held up like a shield for someone else. Laughter is how they refuse to be beaten. What they fear most is the moment the joke stops working.</t>
+  </si>
+  <si>
+    <t>The Naïf</t>
+  </si>
+  <si>
+    <t>The Naïf meets the world as if seeing it for the first time, and gets it gloriously wrong. Like Mr Bean at war with a Christmas turkey, they take on ordinary things with total seriousness and turn them into chaos. They never mean to be funny, which is exactly why they are. People love them because they show how strange our rules really are. Their nightmare is being bored, or, worse, being told to sit still and behave.</t>
+  </si>
+  <si>
+    <t>The naughty little tease you can't help but love - they relish the effect they have on you</t>
+  </si>
+  <si>
+    <t>Dita Von Teese</t>
+  </si>
+  <si>
+    <t>The Tease knows that the best part is the wait. Like Dita Von Teese, who turned burlesque back into an art of glamour and patience, they give away a little, hold back the rest and enjoy every second of the effect. Nothing about it is crude. It is play, done with style, and it leaves everyone smiling. The flat room where nobody is paying attention, and the moment the spell turns into routine, are what they fear.</t>
+  </si>
+  <si>
+    <t>Cheeky, mischievous and with a wicked sense of humour</t>
+  </si>
+  <si>
+    <t>The Elf or Imp is trouble people let in on purpose. They swap the sugar for salt, hide the keys somewhere impossible, pull a coin from behind an ear and look utterly innocent while everyone works out what happened. Their mischief works like a small spell, and suddenly an ordinary Tuesday feels enchanted. It never goes too far, because the point is the grin, not the victim. A house where nothing unexpected ever happens would drive them mad.</t>
+  </si>
+  <si>
+    <t>Russell Brand</t>
+  </si>
+  <si>
+    <t>The Scandalmonger says the unsayable to see what happens next. They poke at taboos, mock the pompous and the pious, and enjoy the gasp as much as the laugh. It can look like shock for its own sake, and sometimes it is. At their best, though, they are testing a room for hypocrisy, daring people to admit what they really think. They would rather be hated than ignored. Boredom and good manners, in that order, are what they fear.</t>
+  </si>
+  <si>
+    <t>The Straight Man is the calm centre that makes the comedy work. Beside Stan Laurel's chaos, Oliver Hardy clings to dignity, and every attempt makes it funnier. This person is the sensible one in the double act of friendship, who holds the plan while others fool around and whose raised eyebrow is the real punchline. They enjoy the fun as much as anyone. They just enjoy running it. What bores them is chaos with nobody to play it against.</t>
+  </si>
+  <si>
+    <t>Full of wisdom and cynicism - able to reflect and comment on the world and show the absurd side of it</t>
+  </si>
+  <si>
+    <t>Stephen Colbert</t>
+  </si>
+  <si>
+    <t>The Cynic laughs because the alternative is despair. They read the news, spot the contradiction and turn it into a line that makes the whole table groan and then nod. Like Stephen Colbert, who played a blowhard pundit so perfectly that the nonsense exposed itself, they use irony to tell the truth. Under the eye-rolls is someone who cares a great deal about what is true. Being bored by lies that everyone pretends to believe is what they cannot stand.</t>
+  </si>
+  <si>
+    <t>Serving to attend to your every need</t>
+  </si>
+  <si>
+    <t>The Geisha makes closeness out of attention. They notice a guest is cold before the guest does, remember how everyone takes their tea and set the table so that each person feels expected. Real geisha are trained artists of conversation, music and timing, and this person has the same gift for making an evening feel effortless. For them it is love in its most practical form. They give generously and rarely ask for anything back. The empty table, care with no one there to receive it, is their loneliest thought.</t>
+  </si>
+  <si>
+    <t>The Muse makes other people want to create. Around them, friends pick up the guitar again, finish the novel, cook something ambitious. In Greek myth the Muses were born of Memory itself, and poets began their work by calling on them. This person inspires through attention and beauty, and creates as much as they inspire, even if their name is rarely on the cover. Their fear is being admired from a distance, loved as an idea rather than known.</t>
+  </si>
+  <si>
+    <t>John McClane</t>
+  </si>
+  <si>
+    <t>The Rough Diamond will never write a poem, but they will drive through the night to be there. In Die Hard, John McClane crawls through air ducts and walks barefoot over broken glass to reach Holly, in a marriage that had run out of words. That is this person: blunt, loyal, better with actions than speeches. The love is unpolished and completely real. What they fear is losing someone because they could never quite say it.</t>
+  </si>
+  <si>
+    <t>The Pleasure Seeker treats life as a feast and people as the best course. Casanova crossed Europe chasing beauty, conversation, cards and romance, and wrote it all down in thousands of pages of memoirs. What is less often told is how it ended: an ageing librarian in a Bohemian castle, reliving every encounter on paper. This person chases delight with real courage. Underneath runs an older fear, that when the music stops they will be alone.</t>
+  </si>
+  <si>
+    <t>Clean cut, saves the day, wins the heart, sweeps you off your feet</t>
+  </si>
+  <si>
+    <t>The Knight in Shining Armour shows love by turning up. At the end of An Officer and a Gentleman, Zack Mayo walks into the factory in dress whites and carries Paula out past the cheering workers. This person loves in grand, decisive gestures and keeps every promise. They protect the people they love fiercely. Beneath the armour is the fear of being unneeded, of arriving in full uniform to find no one waiting.</t>
+  </si>
+  <si>
+    <t>The Pure Heart</t>
+  </si>
+  <si>
+    <t>The Pure Heart loves without games: no strategy, no keeping score, no pretending to care less than they do. Like Romeo and Juliet at the balcony, they fall completely and believe love should be enough to overcome anything. It makes them tender and trusting, and easy to hurt. They would rather be hurt than become guarded. Being alone in a world with no one to love that simply is what frightens them.</t>
+  </si>
+  <si>
+    <t>The Flirt makes connection into a game worth playing. A glance, a tease, a joke held a beat too long, and suddenly there is a spark in the room and everyone feels a little more attractive. Betty Boop was drawn that way, all wink and giggle. The fun is the point, but it is also a way of reaching people without risking too much. The room where nobody plays back is the one they dread.</t>
+  </si>
+  <si>
+    <t>The Charmer draws people in by never showing everything. Like Zorro behind the mask, they reveal just enough to make others lean closer: a look, a secret, a flourish, and then they're gone. They have a gift for making someone feel chosen. The mystery isn't a trick for its own sake. It protects a heart that wants closeness badly and is afraid of being seen too clearly, and then left. So they keep one card hidden, always.</t>
+  </si>
+  <si>
+    <t>The Bad Influence</t>
+  </si>
+  <si>
+    <t>Courtney Love</t>
+  </si>
+  <si>
+    <t>The Bad Influence is the reason the evening got interesting. They suggest the midnight swim, the last-minute concert, the road trip nobody planned, and somehow everyone says yes. Like Courtney Love on stage, they are loud, raw and unapologetic about what they feel, and they would never trade intensity for politeness. The rebellion isn't cruelty. It is their way of saying: be real with me. The one thing they won't allow is being tamed into someone safe, and then left for being boring.</t>
+  </si>
+  <si>
+    <t>Marilyn Monroe</t>
+  </si>
+  <si>
+    <t>The Sex Symbol knows exactly what effect they have and how to use it. They walk into a room and the room rearranges itself. Marilyn Monroe built that power herself, from the voice to the walk, and then set up her own production company to take back a career the studio wanted to own. Yet by many accounts the woman the whole world desired was deeply lonely. That is this person's secret: wanted by everyone, known by very few.</t>
+  </si>
+  <si>
+    <t>The Romantic falls in love with beauty itself, and then tries to understand it. Byron could write 'She walks in beauty, like the night' and spend the rest of a short, restless life chasing what it meant. This person reads, reflects and writes the long letter instead of the quick message. Love, for them, is a way of knowing the world more deeply. What they dread is shallow company, to be surrounded by people and still unseen.</t>
+  </si>
+  <si>
+    <t>The Fairy Godparent</t>
+  </si>
+  <si>
+    <t>Always there mysteriously caring for you. Looking out for you behind the scenes</t>
+  </si>
+  <si>
+    <t>Fairy Godmother in Cinderella</t>
+  </si>
+  <si>
+    <t>The Fairy Godparent changes lives from the wings. Like Cinderella's fairy godmother, who turns a pumpkin into a carriage and then slips quietly away, they work the magic and let someone else go to the ball. They notice what a friend needs before it is said, pull strings nobody sees and never ask for thanks. Their one rule is that the spell must help and never harm. What they fear is meddling, a kindness that goes wrong at midnight.</t>
+  </si>
+  <si>
+    <t>The Genie makes something out of nothing. Ask for help with a party, a speech or a broken heart and they arrive in a burst of ideas, jokes and energy, turning the request into more than anyone imagined. Like Aladdin's genie, with phenomenal cosmic power and an itty-bitty living space, they spend so much time granting wishes that no one thinks to ask what they want. Their own secret wish is freedom. Their fear is a wish granted too literally, with results nobody wanted.</t>
+  </si>
+  <si>
+    <t>The Entertainer always has a coin behind someone's ear. At a kitchen table or a bus stop, out comes a pack of cards, and for one minute the ordinary world goes strange and everyone is a child again. It is everyday magic, and it is for everyone. They practise for hours so that the trick looks effortless, and the reward is a stranger's gasp turning into a laugh. The trick that fails, the moment that falls flat, is what keeps them practising.</t>
+  </si>
+  <si>
+    <t>The Alchemist believes almost anything can become something better with patience and the right combination. They experiment, fail, adjust and try again, keeping notes nobody else can read. Legend made Nicolas Flamel the finder of the philosopher's stone, though the real Flamel was a Paris scribe and the story grew up long after his death, which shows how badly people want this kind of magic to be true. What they fear is a result they can't undo.</t>
+  </si>
+  <si>
+    <t>The Good Wizard has a gift and a duty, and knows which matters more. Like Harry Potter, they discover that they can do extraordinary things, then spend years learning that power only counts when it protects someone. They step in when hope is running out and turn fear into a plan. Making things right is what drives them. What haunts them is the spell that goes wrong, and the friend they could not save.</t>
+  </si>
+  <si>
+    <t>The Sorcerer's Apprentice has just discovered what they can do and can't wait to do all of it. Like Mickey in Fantasia, they borrow the master's hat, bring a broom to life to fetch the water, then watch in horror as the brooms multiply and the room floods. It is the oldest lesson in magic: power grows faster than wisdom. This person learns it with enthusiasm and a few mishaps. That flood, a spell they can't stop, is exactly what they fear.</t>
+  </si>
+  <si>
+    <t>The Illusionist loves the moment someone's certainty wobbles. Like M.C. Escher, with staircases that climb forever and hands that draw each other, they build puzzles for the mind and enjoy watching people fall in. It is play with a purpose, because after the trick everyone sees a little differently. They are never quite what they seem, and they like it that way. Being figured out completely, with no surprises left, would be the end of the fun.</t>
+  </si>
+  <si>
+    <t>The Siren changes the air in a room. People find themselves drawn in without quite knowing why, the way sailors in the old myths steered towards a song they could not resist. This person's allure is real and they know it, which is exactly why they handle it with care. Attraction, for them, is a power that can transform someone or wreck them. Their fear is the spell that works too well, and the harm it does.</t>
+  </si>
+  <si>
+    <t>Loki</t>
+  </si>
+  <si>
+    <t>The Trickster breaks rules to show they were never as solid as everyone thought. Like Loki in the Norse myths, they play pranks on the powerful, turn a situation inside out and leave the gods themselves arguing. Nothing they do is an accident. Behind the mischief is a point: certainty is a kind of prison, and someone has to pick the lock. Being caught before the trick has done its work is what they fear.</t>
+  </si>
+  <si>
+    <t>The Omnipotent One</t>
+  </si>
+  <si>
+    <t>Sistine Chapel</t>
+  </si>
+  <si>
+    <t>The Omnipotent One likes to hold the whole picture. Like the figure on the Sistine Chapel ceiling reaching out to give Adam life, they want to make the world and set it in order. They are the one who plans the trip, runs the project and knows how every piece fits, and when it works, it feels like magic. Surprise is what they fear most, the one piece that moves on its own and undoes everything they set up.</t>
+  </si>
+  <si>
+    <t>The Clairvoyant seems to know how things will turn out before anyone else. Like Gandalf, who senses early that even Gollum still has some part to play, they read people and patterns and see several moves ahead. Their advice can sound mysterious because it rests on things others haven't noticed yet. They change situations by understanding them first. What keeps them awake is the thing they failed to foresee.</t>
+  </si>
+  <si>
+    <t>Roald Dahl's BFG</t>
+  </si>
+  <si>
+    <t>The Gentle Giant is strong enough to frighten anyone and chooses to be kind. Like Roald Dahl's BFG, the one giant who refuses to eat children and instead blows good dreams through their windows, they break with their own kind to protect the small. Tenderness is how they rebel. They stand up to bullies, and rarely need to raise their voice to do it. Their fear is being powerless to protect someone smaller than them.</t>
+  </si>
+  <si>
+    <t>The Rule Breaker makes new things by refusing permission. Banksy paints on walls that belong to other people, and once had a framed painting shred itself the moment it sold at auction. This person hacks the familiar to show what is wrong with it, and leaves something better in the crack. They create to set things free, themselves included. Being bought, framed and hung on the establishment's wall is their idea of defeat.</t>
+  </si>
+  <si>
+    <t>They know the deal, they call the shots, they make the rules.</t>
+  </si>
+  <si>
+    <t>The Gangster lives by a code, not by the law. Their loyalty goes to the crew, the family, the neighbourhood, and they protect their own fiercely. Al Capone ran a soup kitchen in Chicago during the Depression while running an empire built on illegal liquor, and plenty of people there saw him as one of their own. This person knows how things really work and makes their own rules. What they fear is being pushed around by a system that never worked for people like them.</t>
+  </si>
+  <si>
+    <t>The Thrill Seeker needs to feel alive, and safe rarely does it. They jump first and check the depth afterwards, turning danger into a game and fear into a laugh with friends. Jackass made a career of it: bruises, stunts and helpless laughter. Behind the recklessness is a hunger for freedom, proof that nobody can fence them in. The padded, sensible life, where nothing happens and nothing is theirs, frightens them more than any drop.</t>
+  </si>
+  <si>
+    <t>They don't play by the rules, but they get results.</t>
+  </si>
+  <si>
+    <t>The Maverick doesn't play by the rules, but they get results, and the results are usually fair. Like Robin Hood, they take from those who have too much, hand it to those who have too little and vanish into the forest before anyone can say thank you. They trust their own code over anyone's orders. They are brave because it matters, not for the applause. Being told to stand by while something unfair happens is what they cannot bear.</t>
+  </si>
+  <si>
+    <t>Peaches Geldof</t>
+  </si>
+  <si>
+    <t>The Adolescent rebels on instinct, because something in the adult world smells false. They dye their hair, slam the door and refuse to be told who to be, and under the noise is a surprisingly pure idea: that life should be more honest than this. They care deeply about what is real and not at all about what is proper. Growing up into someone they would despise is the future they refuse.</t>
+  </si>
+  <si>
+    <t>The Subverter uses a joke like a crowbar. They mock what everyone else treats as sacred and grin while they do it, until the comfortable start to squirm and the room has to think again. The Joker is the dark extreme of this, laughter as chaos. Most Subverters are far kinder: satirists who unsettle power so that something freer can get in. Being silenced, the joke taken away, is what they fear.</t>
+  </si>
+  <si>
+    <t>The Fugitive loves like a getaway. Passion, for them, means choosing someone against the world: two people in a car, the road ahead and no way back. Bonnie and Clyde became the legend of it, and Bonnie wrote poems predicting how it would end. This person is swept away by love and by freedom at once, and often can't tell the two apart. Getting caught, pinned down and made to settle is the ending they keep running from.</t>
+  </si>
+  <si>
+    <t>Uproots order, embraces chaos because they know it needs to happen for things to change.</t>
+  </si>
+  <si>
+    <t>The Disrupter knows that some things must be broken before they can be rebuilt. In Hindu tradition Shiva dances the world to its end so that it can begin again, and this person carries a small spark of that fire. They shake up the team, the habit, the relationship gone stale, not out of anger but because change is overdue. What they fear is the slow decay of things nobody dares to touch.</t>
+  </si>
+  <si>
+    <t>Sparking off the new and controlling it as it grows.</t>
+  </si>
+  <si>
+    <t>The Leading Edge spots the rebellion before it has a name, then shapes it. Malcolm McLaren put together the Sex Pistols, dressed them from the King's Road shop he ran with Vivienne Westwood and turned punk from a mood into a movement. This person is part rebel, part strategist: they love the new and they like to steer it. What worries them is losing the wheel, watching the thing they started run off without them or get tamed by the mainstream.</t>
+  </si>
+  <si>
+    <t>The Devil's Advocate argues the other side, on purpose. The name comes from an old office of the Catholic Church whose holder had to make the case against anyone proposed for sainthood. This person tests every idea by pushing hard against it, because an idea that can't survive the argument isn't worth believing. People find them exhausting and later realise they were right to ask. Their fear is the room where everyone nods and no one is allowed to think.</t>
+  </si>
+  <si>
+    <t>The Caring Leader holds authority lightly and uses it to protect. They listen first, set clear boundaries and stay calm when everyone else is shouting, so that people feel safe enough to do their best. Gandhi moved millions with little more than a spinning wheel, a walking stick and fierce self-discipline. This person's power comes from the trust they earn. Chaos breaking out on their watch, and the people in their care hurt by it, is their deepest fear.</t>
+  </si>
+  <si>
+    <t>The Perfectionist sees the finished thing before anyone else does, then shapes every detail until it matches. Like Anna Wintour deciding what the world will wear next, they rule by taste, and their standards become the law of the room. It can look cold. In truth they care intensely, and mediocrity feels to them like a small disorder, a crack in the world. Their fear is losing control of the result and watching something careless go out with their name on it.</t>
+  </si>
+  <si>
+    <t>The People's Representative holds power without leaving the people behind. At the 1995 Rugby World Cup final, Nelson Mandela walked onto the pitch in a Springbok jersey, the shirt of a team many Black South Africans had long seen as a symbol of apartheid, and a divided stadium chanted 'Nelson! Nelson!' This person leads by belonging. They speak plainly, show up and make everyone feel part of it. Division, a country, a team or a family pulling apart, is what they fear.</t>
+  </si>
+  <si>
+    <t>The Reformer uses power to open doors. They respect what works and are willing to tear down what doesn't, rebuilding the system so that more people can live freely inside it. Abraham Lincoln held a divided country together through a civil war and used the presidency to end slavery. This person governs with the future in mind. What keeps them careful is the fear of chaos, the whole structure collapsing while they are trying to change it.</t>
+  </si>
+  <si>
+    <t>The Noble Ruler</t>
+  </si>
+  <si>
+    <t>The Noble Ruler leads the way the old legends say rulers should. Like King Arthur at the Round Table, where no seat stands higher than another, they give everyone a place and ask only that each keeps their word. They take the hard decisions, carry the weight of other people's safety and stand in front when trouble comes. Duty is how they love. Their fear is disorder breaking into what they have built, and failing the people who trusted them.</t>
+  </si>
+  <si>
+    <t>The Diva knows exactly how things should be and sees no reason to accept less. The lighting, the table, the song: it must be right, and they will say so. People call it demanding. Underneath is something almost childlike, a pure belief that life should be beautiful and that someone ought to insist on it. Mariah Carey has spent decades turning that insistence into an art form. Being ignored, and watching everything slide into a mess, is what they cannot stand.</t>
+  </si>
+  <si>
+    <t>The Charismatic Leader makes being in charge look like fun. The story goes that Richard Branson got into the airline business after a cancelled flight left him stranded, and he has since crossed oceans by balloon and turned up to launches in costume. This person leads with jokes, big gestures and a sense of adventure, and people follow because it is exciting to. Still, they are in charge. The show falling into chaos, or, almost as bad, turning dull, is what they fear.</t>
+  </si>
+  <si>
+    <t>The Magnetic Leader leads up close. They remember names, hold eye contact a second longer and make each person feel like the only one in the room. That was said of Bill Clinton for decades, a politician who could also pick up a saxophone and win the night. This person rules through warmth and charm, and knows exactly how well it works. Losing the room is their nightmare, the moment the spell breaks and order goes with it.</t>
+  </si>
+  <si>
+    <t>The ruler who changed everything.</t>
+  </si>
+  <si>
+    <t>The Legend is the one people remember when everything was shaking. Winston Churchill spent years dismissed and out of favour before 1940, when his speeches held a frightened country together. This person turns crises into turning points by force of will and the right words at the right time. They think in decades, not days. Their fear is chaos winning, and history remembering them as the one who let it.</t>
+  </si>
+  <si>
+    <t>Leading the way in challenging the status quo.</t>
+  </si>
+  <si>
+    <t>The Revolutionary builds power by tearing down the old order. Che Guevara went from medical student to guerrilla commander to president of Cuba's national bank, where he signed the banknotes simply 'Che'. This person leads with conviction and symbols, and refuses to compromise. The irony they carry is that, once they have won, they fear the next revolution as much as any king did. Order was what they wanted all along, as long as it was theirs.</t>
+  </si>
+  <si>
+    <t>The Judge brings order by getting to the truth. They listen to both sides, cut through the noise, weigh what is real and decide, then stand by the decision. Judge Judy made a television career out of doing it briskly and without apology. Fairness matters more to them than being liked, and they believe clear rules protect people. What they fear is chaos dressed up as kindness, and the lie that nobody bothered to check.</t>
+  </si>
+  <si>
+    <t>Passes on their knowledge and supports others in their challenges</t>
+  </si>
+  <si>
+    <t>The Mentor turns what they know into someone else's courage. They listen properly, ask the question that makes the penny drop and give advice that is honest without being harsh. Oprah Winfrey built a career on exactly that kind of conversation, helping millions of people think more clearly about their own lives. This person is happiest when a student outgrows them. Steering someone wrong, with advice that turns out to be false, is what they would never forgive themselves for.</t>
+  </si>
+  <si>
+    <t>The Architect sees how the pieces fit before any of them exist. Give them a mess, a kitchen, a company, a holiday for twelve, and they will draw the plan, test it in their head and build it so that it stands. Knowledge, for them, is something to build with. They love precision and cannot abide a structure that only looks sound. The hidden flaw, the beam that was never really load-bearing, is what they fear.</t>
+  </si>
+  <si>
+    <t>The Dude has worked out that most of life's drama isn't worth the fuss. In The Big Lebowski everyone around the Dude is scheming, shouting and lying, and all the Dude wants is the rug back, the one that really tied the room together. Everything this person knows was learned by living, and it comes down to this: stay easy, keep it real, don't take the bait. They lower the temperature wherever they go. Being dragged into other people's lies is what they dread.</t>
+  </si>
+  <si>
+    <t>The Philosopher can't leave a question alone. Why do we believe this? What would it mean if it were not true? Plato set down his ideas as conversations, most famously the Symposium, a dinner where friends argue about love until dawn. This person thinks in company and in solitude, and travels furthest without leaving the chair. The truth is always one layer deeper for them. Being fooled by an easy answer is what they fear.</t>
+  </si>
+  <si>
+    <t>The Grandmaster</t>
+  </si>
+  <si>
+    <t>The Grandmaster wins by seeing further. At the board or in life, they stay calm while others rush, read the whole position and choose the move that will matter ten moves from now. They are brave in a patient way, willing to give up a piece to win the game. Chess players call it understanding the position. This person calls it paying attention. What they fear is the trap they didn't see.</t>
+  </si>
+  <si>
+    <t>The Prodigy knew things early and still wants to know everything. They were reading the grown-up books at ten and asking questions that silenced the dinner table, and the delight never went out of it. Tavi Gevinson was writing a fashion blog read around the world before she was a teenager. This person has a mind that runs ahead with wide-open eyes. Being patronised, or discovering that the grown-ups were bluffing, is what they fear.</t>
+  </si>
+  <si>
+    <t>A wise soul who reveals the truth using humour and the absurd to show how things really are.</t>
+  </si>
+  <si>
+    <t>The Fool in King Lear</t>
+  </si>
+  <si>
+    <t>The Wise Fool tells the truth sideways. In King Lear it is the Fool, the one member of the court allowed to mock the king, who sees most clearly the mess Lear has made. This person uses jokes, riddles and absurdity to slip past people's defences, because the truth goes down easier with a laugh. They are cleverer than they let on. Their fear is a world full of lies that nobody dares to laugh at.</t>
+  </si>
+  <si>
+    <t>The Connoisseur studies what they love until they can say why it is good. They taste slowly, notice the detail others miss and find the words for it, and the words make the pleasure deeper, not colder. A sommelier does it with a glass. This person does it with music, food, people and places. Knowing is how they love. Their fear is being fooled by the fake label or the flattering story, because a pleasure built on a lie is spoiled.</t>
+  </si>
+  <si>
+    <t>The Game-Changer turns understanding into transformation. They study a problem until they see what everyone else missed, then make it so simple it seems obvious. In 2007 Steve Jobs walked onto a stage with a phone that made every other phone look old. This person isn't content to know things; they want the knowledge to change how people live. Getting it wrong at scale, a revolution built on a flawed idea, is what frightens them.</t>
+  </si>
+  <si>
+    <t>The Lone Voice says what they have found, even when everyone important wants them to stop. Galileo turned his telescope on Jupiter, saw moons circling it and knew the Earth was not the centre of everything, and he kept saying so until the Church put him on trial and forced him to take it back. This person values evidence over approval, and loneliness is often the price. Their fear is a comfortable lie becoming the official truth.</t>
+  </si>
+  <si>
+    <t>The Scientist trusts only what can be tested. Marie Curie worked for years in a leaking shed, processing tonnes of ore by hand to isolate radium, and won Nobel prizes in two different sciences. This person measures carefully, writes everything down and follows the evidence even when it is inconvenient. Rigour is how they keep a messy world in order. The result that turns out to be false is the one that haunts them.</t>
+  </si>
+  <si>
+    <t>The One Next Door</t>
+  </si>
+  <si>
+    <t>Simple, down to earth, polite - the kind of person your family would love you to bring home for tea</t>
+  </si>
+  <si>
+    <t>A down-to-earth rogue who can get away with anything</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freedom
+Independence 
+Bravery 
+Self-sufficiency</t>
+  </si>
+  <si>
+    <t>The Explorer archetype encourages freedom, adventure and self-discovery. Explorer is appealing to the consumer's desire for new experiences and challenge them to break free from the mundane. He is restless and adventurous, always seeking new horizons and experiences beyond the familiar.</t>
+  </si>
+  <si>
+    <t>The Explorer archetype encourages freedom, adventure and self-discovery. Explorer is appealing to the consumer's desire for new experiences and challenge them to break free from the mundane. The Explorer is restless and adventurous, always seeking new horizons and experiences beyond the familiar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mastery
+Courage 
+Strength
+Perseverence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mastery
+Courage 
+Strength
+Perseverance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety
+Sense of wonder
+Trust 
+Honesty </t>
+  </si>
+  <si>
+    <t>The Innocent archetype represents purity and the reach for perfection. Optimistic and honest, innocent brands are often associated with health, beauty, and organic products with the aim to be simple, positive, and genuine, therfore evoking a sense of trust and safety​.</t>
+  </si>
+  <si>
+    <t>The Innocent archetype represents purity and the reach for perfection. Optimistic and honest, innocent brands are often associated with health, beauty, and organic products with the aim to be simple, positive, and genuine, therefore evoking a sense of trust and safety​.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pleasure
+Enjoyment 
+Humor 
+Originality </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Jester archetype is all about fun and humour. Brands like this want to bring joy and are characterized by their playful and light-hearted nature. Jester personality is engaging, invoking happiness and laughter, often seen in confectionary or entertainment industries​ - and using 2sc degree to make messages more appreciable. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Jester archetype is all about fun and humour. Brands like this want to bring joy and are characterized by their playful and light-hearted nature. Jester personality is engaging, invoking happiness and laughter, often seen in confectionary or entertainment industries​ - and using irony and tongue-in-cheek humour to make messages more likeable. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isolation
+Loneliness
+Coldness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Lover archetype embodies passion, intimacy, and commitment. Lovers personalities generally use messaging that promotes enjoyment of life's pleasures, builds relationships, and encourages customers to follow their passions and fields of interest. All about feeling good. </t>
+  </si>
+  <si>
+    <t>The sage archetype seeks knowledge and truth. Sage focus on wisdom, intelligence, and the sharing of knowledge, appealing to the customer's intellectual side​. The Sage can be seen as a guide or mentor, and aims to understand the world deeply.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traditional and clean fonts that suggest wisdom and clarity.
+Libre Baskerville for its readability and academic look.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service
+Compassion
+Patience
+Empathy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The caregiver archetype aims to be nurturing and protective. It focuses on service and support. The Caregiver's personality conveys trust, comfort, and a sense of caring for others, aiming to make customers feel safe and cared for​. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bright, bold colors that inspire creativity or monochromatic schemes that suggest customizability
+Examples: vibrant teals (#00B8A9), purples (#6A0572), and oranges (#FF6107).</t>
   </si>
 </sst>
 </file>
@@ -4355,7 +4908,7 @@
         <v>20</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>21</v>
+        <v>1159</v>
       </c>
       <c r="J5" s="9" t="s">
         <v>22</v>
@@ -4448,13 +5001,13 @@
         <v>39</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>40</v>
+        <v>1142</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>41</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>42</v>
+        <v>1144</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>43</v>
@@ -4502,7 +5055,7 @@
         <v>51</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>52</v>
+        <v>1146</v>
       </c>
       <c r="E8" s="15" t="s">
         <v>53</v>
@@ -4556,13 +5109,13 @@
         <v>39</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>63</v>
+        <v>1147</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>64</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>65</v>
+        <v>1149</v>
       </c>
       <c r="G9" s="9" t="s">
         <v>66</v>
@@ -4610,13 +5163,13 @@
         <v>27</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>74</v>
+        <v>1150</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>75</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>76</v>
+        <v>1152</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>77</v>
@@ -4667,10 +5220,10 @@
         <v>85</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>86</v>
+        <v>1153</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>87</v>
+        <v>1154</v>
       </c>
       <c r="G11" s="9" t="s">
         <v>88</v>
@@ -4886,7 +5439,7 @@
         <v>130</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>131</v>
+        <v>1155</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>132</v>
@@ -4898,7 +5451,7 @@
         <v>134</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>135</v>
+        <v>1156</v>
       </c>
       <c r="K15" s="9" t="s">
         <v>136</v>
@@ -4934,13 +5487,13 @@
         <v>15</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>140</v>
+        <v>1157</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>141</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>142</v>
+        <v>1158</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>143</v>
@@ -9353,10 +9906,10 @@
         <v>84</v>
       </c>
       <c r="G32" s="46" t="s">
-        <v>342</v>
+        <v>1139</v>
       </c>
       <c r="H32" s="43" t="s">
-        <v>343</v>
+        <v>1140</v>
       </c>
       <c r="I32" s="43" t="s">
         <v>680</v>
@@ -9446,7 +9999,7 @@
         <v>352</v>
       </c>
       <c r="H34" s="43" t="s">
-        <v>353</v>
+        <v>1141</v>
       </c>
       <c r="I34" s="43" t="s">
         <v>354</v>
@@ -9581,13 +10134,13 @@
         <v>372</v>
       </c>
       <c r="H37" s="43" t="s">
-        <v>373</v>
+        <v>983</v>
       </c>
       <c r="I37" s="43" t="s">
-        <v>374</v>
+        <v>984</v>
       </c>
       <c r="J37" s="26" t="s">
-        <v>681</v>
+        <v>985</v>
       </c>
       <c r="K37" s="95" t="s">
         <v>682</v>
@@ -9632,7 +10185,7 @@
         <v>378</v>
       </c>
       <c r="J38" s="26" t="s">
-        <v>684</v>
+        <v>986</v>
       </c>
       <c r="K38" t="s">
         <v>685</v>
@@ -9677,7 +10230,7 @@
         <v>381</v>
       </c>
       <c r="J39" s="26" t="s">
-        <v>687</v>
+        <v>987</v>
       </c>
       <c r="K39" t="s">
         <v>688</v>
@@ -9722,7 +10275,7 @@
         <v>384</v>
       </c>
       <c r="J40" s="26" t="s">
-        <v>690</v>
+        <v>988</v>
       </c>
       <c r="K40" s="95" t="s">
         <v>691</v>
@@ -9767,7 +10320,7 @@
         <v>387</v>
       </c>
       <c r="J41" s="26" t="s">
-        <v>693</v>
+        <v>989</v>
       </c>
       <c r="K41" t="s">
         <v>694</v>
@@ -9809,10 +10362,10 @@
         <v>389</v>
       </c>
       <c r="I42" s="43" t="s">
-        <v>390</v>
+        <v>990</v>
       </c>
       <c r="J42" s="26" t="s">
-        <v>696</v>
+        <v>991</v>
       </c>
       <c r="K42" t="s">
         <v>697</v>
@@ -9851,13 +10404,13 @@
         <v>391</v>
       </c>
       <c r="H43" s="43" t="s">
-        <v>392</v>
+        <v>992</v>
       </c>
       <c r="I43" s="43" t="s">
         <v>393</v>
       </c>
       <c r="J43" s="26" t="s">
-        <v>699</v>
+        <v>993</v>
       </c>
       <c r="K43" t="s">
         <v>700</v>
@@ -9902,7 +10455,7 @@
         <v>396</v>
       </c>
       <c r="J44" s="26" t="s">
-        <v>702</v>
+        <v>994</v>
       </c>
       <c r="K44" t="s">
         <v>703</v>
@@ -9947,7 +10500,7 @@
         <v>399</v>
       </c>
       <c r="J45" s="26" t="s">
-        <v>705</v>
+        <v>995</v>
       </c>
       <c r="K45" t="s">
         <v>706</v>
@@ -9983,16 +10536,16 @@
         <v>117</v>
       </c>
       <c r="G46" s="46" t="s">
-        <v>400</v>
+        <v>996</v>
       </c>
       <c r="H46" s="43" t="s">
         <v>401</v>
       </c>
       <c r="I46" s="43" t="s">
-        <v>402</v>
+        <v>997</v>
       </c>
       <c r="J46" s="26" t="s">
-        <v>708</v>
+        <v>998</v>
       </c>
       <c r="K46" t="s">
         <v>709</v>
@@ -10037,7 +10590,7 @@
         <v>405</v>
       </c>
       <c r="J47" s="26" t="s">
-        <v>711</v>
+        <v>999</v>
       </c>
       <c r="K47" t="s">
         <v>712</v>
@@ -10073,16 +10626,16 @@
         <v>139</v>
       </c>
       <c r="G48" s="46" t="s">
-        <v>408</v>
+        <v>1000</v>
       </c>
       <c r="H48" s="43" t="s">
-        <v>409</v>
+        <v>1001</v>
       </c>
       <c r="I48" s="43" t="s">
         <v>410</v>
       </c>
       <c r="J48" t="s">
-        <v>714</v>
+        <v>1002</v>
       </c>
       <c r="K48" t="s">
         <v>715</v>
@@ -10127,7 +10680,7 @@
         <v>414</v>
       </c>
       <c r="J49" t="s">
-        <v>717</v>
+        <v>1003</v>
       </c>
       <c r="K49" t="s">
         <v>718</v>
@@ -10163,16 +10716,16 @@
         <v>26</v>
       </c>
       <c r="G50" s="46" t="s">
-        <v>415</v>
+        <v>1004</v>
       </c>
       <c r="H50" s="43" t="s">
-        <v>416</v>
+        <v>1005</v>
       </c>
       <c r="I50" s="43" t="s">
-        <v>417</v>
+        <v>1006</v>
       </c>
       <c r="J50" t="s">
-        <v>720</v>
+        <v>1007</v>
       </c>
       <c r="K50" t="s">
         <v>721</v>
@@ -10211,13 +10764,13 @@
         <v>418</v>
       </c>
       <c r="H51" s="43" t="s">
-        <v>419</v>
+        <v>1008</v>
       </c>
       <c r="I51" s="43" t="s">
         <v>420</v>
       </c>
       <c r="J51" t="s">
-        <v>723</v>
+        <v>1009</v>
       </c>
       <c r="K51" t="s">
         <v>724</v>
@@ -10256,13 +10809,13 @@
         <v>421</v>
       </c>
       <c r="H52" s="43" t="s">
-        <v>422</v>
+        <v>1010</v>
       </c>
       <c r="I52" s="43" t="s">
         <v>423</v>
       </c>
       <c r="J52" t="s">
-        <v>726</v>
+        <v>1011</v>
       </c>
       <c r="K52" t="s">
         <v>727</v>
@@ -10298,7 +10851,7 @@
         <v>73</v>
       </c>
       <c r="G53" s="46" t="s">
-        <v>424</v>
+        <v>1012</v>
       </c>
       <c r="H53" s="43" t="s">
         <v>425</v>
@@ -10307,7 +10860,7 @@
         <v>426</v>
       </c>
       <c r="J53" t="s">
-        <v>729</v>
+        <v>1013</v>
       </c>
       <c r="K53" t="s">
         <v>730</v>
@@ -10346,13 +10899,13 @@
         <v>427</v>
       </c>
       <c r="H54" s="43" t="s">
-        <v>428</v>
+        <v>1014</v>
       </c>
       <c r="I54" s="43" t="s">
         <v>429</v>
       </c>
       <c r="J54" t="s">
-        <v>732</v>
+        <v>1015</v>
       </c>
       <c r="K54" t="s">
         <v>733</v>
@@ -10397,7 +10950,7 @@
         <v>432</v>
       </c>
       <c r="J55" t="s">
-        <v>735</v>
+        <v>1016</v>
       </c>
       <c r="K55" t="s">
         <v>736</v>
@@ -10439,10 +10992,10 @@
         <v>434</v>
       </c>
       <c r="I56" s="43" t="s">
-        <v>948</v>
+        <v>1017</v>
       </c>
       <c r="J56" t="s">
-        <v>738</v>
+        <v>1018</v>
       </c>
       <c r="K56" t="s">
         <v>739</v>
@@ -10484,10 +11037,10 @@
         <v>436</v>
       </c>
       <c r="I57" s="43" t="s">
-        <v>437</v>
+        <v>1019</v>
       </c>
       <c r="J57" t="s">
-        <v>741</v>
+        <v>1020</v>
       </c>
       <c r="K57" t="s">
         <v>742</v>
@@ -10532,7 +11085,7 @@
         <v>440</v>
       </c>
       <c r="J58" t="s">
-        <v>744</v>
+        <v>1021</v>
       </c>
       <c r="K58" t="s">
         <v>745</v>
@@ -10568,7 +11121,7 @@
         <v>139</v>
       </c>
       <c r="G59" s="46" t="s">
-        <v>443</v>
+        <v>1022</v>
       </c>
       <c r="H59" s="43" t="s">
         <v>444</v>
@@ -10577,7 +11130,7 @@
         <v>747</v>
       </c>
       <c r="J59" s="26" t="s">
-        <v>748</v>
+        <v>1023</v>
       </c>
       <c r="K59" t="s">
         <v>749</v>
@@ -10616,13 +11169,13 @@
         <v>445</v>
       </c>
       <c r="H60" s="43" t="s">
-        <v>982</v>
+        <v>1024</v>
       </c>
       <c r="I60" s="43" t="s">
         <v>446</v>
       </c>
       <c r="J60" t="s">
-        <v>751</v>
+        <v>1025</v>
       </c>
       <c r="K60" t="s">
         <v>752</v>
@@ -10667,7 +11220,7 @@
         <v>449</v>
       </c>
       <c r="J61" t="s">
-        <v>754</v>
+        <v>1026</v>
       </c>
       <c r="K61" t="s">
         <v>755</v>
@@ -10709,10 +11262,10 @@
         <v>451</v>
       </c>
       <c r="I62" s="43" t="s">
-        <v>452</v>
+        <v>1027</v>
       </c>
       <c r="J62" t="s">
-        <v>757</v>
+        <v>1028</v>
       </c>
       <c r="K62" t="s">
         <v>758</v>
@@ -10757,7 +11310,7 @@
         <v>455</v>
       </c>
       <c r="J63" t="s">
-        <v>760</v>
+        <v>1029</v>
       </c>
       <c r="K63" t="s">
         <v>761</v>
@@ -10802,7 +11355,7 @@
         <v>458</v>
       </c>
       <c r="J64" t="s">
-        <v>763</v>
+        <v>1030</v>
       </c>
       <c r="K64" t="s">
         <v>764</v>
@@ -10847,7 +11400,7 @@
         <v>460</v>
       </c>
       <c r="J65" t="s">
-        <v>767</v>
+        <v>1031</v>
       </c>
       <c r="K65" t="s">
         <v>768</v>
@@ -10892,7 +11445,7 @@
         <v>463</v>
       </c>
       <c r="J66" t="s">
-        <v>770</v>
+        <v>1032</v>
       </c>
       <c r="K66" t="s">
         <v>771</v>
@@ -10937,7 +11490,7 @@
         <v>466</v>
       </c>
       <c r="J67" t="s">
-        <v>773</v>
+        <v>1033</v>
       </c>
       <c r="K67" t="s">
         <v>774</v>
@@ -10982,7 +11535,7 @@
         <v>469</v>
       </c>
       <c r="J68" t="s">
-        <v>776</v>
+        <v>1034</v>
       </c>
       <c r="K68" t="s">
         <v>777</v>
@@ -11021,13 +11574,13 @@
         <v>470</v>
       </c>
       <c r="H69" s="43" t="s">
-        <v>471</v>
+        <v>1035</v>
       </c>
       <c r="I69" s="43" t="s">
         <v>472</v>
       </c>
       <c r="J69" t="s">
-        <v>779</v>
+        <v>1036</v>
       </c>
       <c r="K69" t="s">
         <v>780</v>
@@ -11066,13 +11619,13 @@
         <v>475</v>
       </c>
       <c r="H70" s="43" t="s">
-        <v>476</v>
+        <v>1037</v>
       </c>
       <c r="I70" s="43" t="s">
         <v>477</v>
       </c>
       <c r="J70" s="26" t="s">
-        <v>782</v>
+        <v>1038</v>
       </c>
       <c r="K70" t="s">
         <v>783</v>
@@ -11117,7 +11670,7 @@
         <v>480</v>
       </c>
       <c r="J71" t="s">
-        <v>785</v>
+        <v>1039</v>
       </c>
       <c r="K71" t="s">
         <v>786</v>
@@ -11162,7 +11715,7 @@
         <v>483</v>
       </c>
       <c r="J72" t="s">
-        <v>788</v>
+        <v>1040</v>
       </c>
       <c r="K72" t="s">
         <v>789</v>
@@ -11204,10 +11757,10 @@
         <v>485</v>
       </c>
       <c r="I73" s="43" t="s">
-        <v>486</v>
+        <v>1041</v>
       </c>
       <c r="J73" t="s">
-        <v>791</v>
+        <v>1042</v>
       </c>
       <c r="K73" t="s">
         <v>792</v>
@@ -11249,10 +11802,10 @@
         <v>488</v>
       </c>
       <c r="I74" s="43" t="s">
-        <v>489</v>
+        <v>1043</v>
       </c>
       <c r="J74" t="s">
-        <v>794</v>
+        <v>1044</v>
       </c>
       <c r="K74" t="s">
         <v>795</v>
@@ -11288,7 +11841,7 @@
         <v>62</v>
       </c>
       <c r="G75" s="46" t="s">
-        <v>490</v>
+        <v>1045</v>
       </c>
       <c r="H75" s="43" t="s">
         <v>491</v>
@@ -11297,7 +11850,7 @@
         <v>492</v>
       </c>
       <c r="J75" t="s">
-        <v>797</v>
+        <v>1046</v>
       </c>
       <c r="K75" t="s">
         <v>798</v>
@@ -11336,13 +11889,13 @@
         <v>493</v>
       </c>
       <c r="H76" s="43" t="s">
-        <v>494</v>
+        <v>1047</v>
       </c>
       <c r="I76" s="43" t="s">
-        <v>495</v>
+        <v>1048</v>
       </c>
       <c r="J76" t="s">
-        <v>800</v>
+        <v>1049</v>
       </c>
       <c r="K76" t="s">
         <v>801</v>
@@ -11381,13 +11934,13 @@
         <v>496</v>
       </c>
       <c r="H77" s="43" t="s">
-        <v>497</v>
+        <v>1050</v>
       </c>
       <c r="I77" s="43" t="s">
         <v>498</v>
       </c>
       <c r="J77" t="s">
-        <v>803</v>
+        <v>1051</v>
       </c>
       <c r="K77" t="s">
         <v>804</v>
@@ -11429,10 +11982,10 @@
         <v>500</v>
       </c>
       <c r="I78" s="43" t="s">
-        <v>501</v>
+        <v>1052</v>
       </c>
       <c r="J78" t="s">
-        <v>806</v>
+        <v>1053</v>
       </c>
       <c r="K78" t="s">
         <v>807</v>
@@ -11477,7 +12030,7 @@
         <v>504</v>
       </c>
       <c r="J79" t="s">
-        <v>809</v>
+        <v>1054</v>
       </c>
       <c r="K79" t="s">
         <v>810</v>
@@ -11516,13 +12069,13 @@
         <v>505</v>
       </c>
       <c r="H80" s="43" t="s">
-        <v>506</v>
+        <v>1055</v>
       </c>
       <c r="I80" s="43" t="s">
-        <v>507</v>
+        <v>1056</v>
       </c>
       <c r="J80" t="s">
-        <v>812</v>
+        <v>1057</v>
       </c>
       <c r="K80" t="s">
         <v>813</v>
@@ -11561,13 +12114,13 @@
         <v>510</v>
       </c>
       <c r="H81" s="43" t="s">
-        <v>511</v>
+        <v>1058</v>
       </c>
       <c r="I81" s="43" t="s">
         <v>512</v>
       </c>
       <c r="J81" s="26" t="s">
-        <v>815</v>
+        <v>1059</v>
       </c>
       <c r="K81" t="s">
         <v>816</v>
@@ -11612,7 +12165,7 @@
         <v>515</v>
       </c>
       <c r="J82" t="s">
-        <v>818</v>
+        <v>1060</v>
       </c>
       <c r="K82" t="s">
         <v>819</v>
@@ -11654,10 +12207,10 @@
         <v>517</v>
       </c>
       <c r="I83" s="43" t="s">
-        <v>518</v>
+        <v>1061</v>
       </c>
       <c r="J83" t="s">
-        <v>821</v>
+        <v>1062</v>
       </c>
       <c r="K83" t="s">
         <v>822</v>
@@ -11702,7 +12255,7 @@
         <v>521</v>
       </c>
       <c r="J84" t="s">
-        <v>824</v>
+        <v>1063</v>
       </c>
       <c r="K84" t="s">
         <v>825</v>
@@ -11741,13 +12294,13 @@
         <v>522</v>
       </c>
       <c r="H85" s="43" t="s">
-        <v>523</v>
+        <v>1064</v>
       </c>
       <c r="I85" s="43" t="s">
         <v>524</v>
       </c>
       <c r="J85" t="s">
-        <v>827</v>
+        <v>1065</v>
       </c>
       <c r="K85" t="s">
         <v>828</v>
@@ -11783,7 +12336,7 @@
         <v>62</v>
       </c>
       <c r="G86" s="46" t="s">
-        <v>525</v>
+        <v>1066</v>
       </c>
       <c r="H86" s="43" t="s">
         <v>526</v>
@@ -11792,7 +12345,7 @@
         <v>527</v>
       </c>
       <c r="J86" t="s">
-        <v>830</v>
+        <v>1067</v>
       </c>
       <c r="K86" t="s">
         <v>831</v>
@@ -11837,7 +12390,7 @@
         <v>530</v>
       </c>
       <c r="J87" t="s">
-        <v>833</v>
+        <v>1068</v>
       </c>
       <c r="K87" t="s">
         <v>834</v>
@@ -11882,7 +12435,7 @@
         <v>533</v>
       </c>
       <c r="J88" t="s">
-        <v>836</v>
+        <v>1069</v>
       </c>
       <c r="K88" t="s">
         <v>837</v>
@@ -11918,16 +12471,16 @@
         <v>106</v>
       </c>
       <c r="G89" s="46" t="s">
-        <v>534</v>
+        <v>1070</v>
       </c>
       <c r="H89" s="43" t="s">
         <v>535</v>
       </c>
       <c r="I89" s="43" t="s">
-        <v>536</v>
+        <v>1071</v>
       </c>
       <c r="J89" t="s">
-        <v>839</v>
+        <v>1072</v>
       </c>
       <c r="K89" t="s">
         <v>840</v>
@@ -11969,10 +12522,10 @@
         <v>538</v>
       </c>
       <c r="I90" s="43" t="s">
-        <v>539</v>
+        <v>1073</v>
       </c>
       <c r="J90" t="s">
-        <v>842</v>
+        <v>1074</v>
       </c>
       <c r="K90" t="s">
         <v>843</v>
@@ -12017,7 +12570,7 @@
         <v>542</v>
       </c>
       <c r="J91" t="s">
-        <v>845</v>
+        <v>1075</v>
       </c>
       <c r="K91" t="s">
         <v>846</v>
@@ -12053,16 +12606,16 @@
         <v>139</v>
       </c>
       <c r="G92" s="46" t="s">
-        <v>545</v>
+        <v>1076</v>
       </c>
       <c r="H92" s="79" t="s">
-        <v>546</v>
+        <v>1077</v>
       </c>
       <c r="I92" s="43" t="s">
-        <v>547</v>
+        <v>1078</v>
       </c>
       <c r="J92" s="26" t="s">
-        <v>850</v>
+        <v>1079</v>
       </c>
       <c r="K92" t="s">
         <v>851</v>
@@ -12107,7 +12660,7 @@
         <v>550</v>
       </c>
       <c r="J93" t="s">
-        <v>853</v>
+        <v>1080</v>
       </c>
       <c r="K93" t="s">
         <v>854</v>
@@ -12152,7 +12705,7 @@
         <v>553</v>
       </c>
       <c r="J94" t="s">
-        <v>856</v>
+        <v>1081</v>
       </c>
       <c r="K94" t="s">
         <v>857</v>
@@ -12197,7 +12750,7 @@
         <v>556</v>
       </c>
       <c r="J95" t="s">
-        <v>859</v>
+        <v>1082</v>
       </c>
       <c r="K95" t="s">
         <v>860</v>
@@ -12242,7 +12795,7 @@
         <v>559</v>
       </c>
       <c r="J96" t="s">
-        <v>862</v>
+        <v>1083</v>
       </c>
       <c r="K96" t="s">
         <v>863</v>
@@ -12287,7 +12840,7 @@
         <v>562</v>
       </c>
       <c r="J97" t="s">
-        <v>865</v>
+        <v>1084</v>
       </c>
       <c r="K97" t="s">
         <v>866</v>
@@ -12332,7 +12885,7 @@
         <v>565</v>
       </c>
       <c r="J98" t="s">
-        <v>868</v>
+        <v>1085</v>
       </c>
       <c r="K98" t="s">
         <v>869</v>
@@ -12377,7 +12930,7 @@
         <v>568</v>
       </c>
       <c r="J99" t="s">
-        <v>871</v>
+        <v>1086</v>
       </c>
       <c r="K99" t="s">
         <v>872</v>
@@ -12419,10 +12972,10 @@
         <v>849</v>
       </c>
       <c r="I100" s="43" t="s">
-        <v>848</v>
+        <v>1087</v>
       </c>
       <c r="J100" t="s">
-        <v>874</v>
+        <v>1088</v>
       </c>
       <c r="K100" t="s">
         <v>875</v>
@@ -12458,16 +13011,16 @@
         <v>117</v>
       </c>
       <c r="G101" s="46" t="s">
-        <v>570</v>
+        <v>1089</v>
       </c>
       <c r="H101" s="80" t="s">
         <v>571</v>
       </c>
       <c r="I101" s="43" t="s">
-        <v>572</v>
+        <v>1090</v>
       </c>
       <c r="J101" t="s">
-        <v>877</v>
+        <v>1091</v>
       </c>
       <c r="K101" t="s">
         <v>878</v>
@@ -12512,7 +13065,7 @@
         <v>575</v>
       </c>
       <c r="J102" t="s">
-        <v>880</v>
+        <v>1092</v>
       </c>
       <c r="K102" t="s">
         <v>881</v>
@@ -12554,10 +13107,10 @@
         <v>579</v>
       </c>
       <c r="I103" s="43" t="s">
-        <v>580</v>
+        <v>1093</v>
       </c>
       <c r="J103" s="26" t="s">
-        <v>883</v>
+        <v>1094</v>
       </c>
       <c r="K103" t="s">
         <v>884</v>
@@ -12602,7 +13155,7 @@
         <v>583</v>
       </c>
       <c r="J104" t="s">
-        <v>886</v>
+        <v>1095</v>
       </c>
       <c r="K104" t="s">
         <v>887</v>
@@ -12641,13 +13194,13 @@
         <v>584</v>
       </c>
       <c r="H105" s="43" t="s">
-        <v>585</v>
+        <v>1096</v>
       </c>
       <c r="I105" s="43" t="s">
         <v>586</v>
       </c>
       <c r="J105" t="s">
-        <v>889</v>
+        <v>1097</v>
       </c>
       <c r="K105" t="s">
         <v>890</v>
@@ -12692,7 +13245,7 @@
         <v>589</v>
       </c>
       <c r="J106" t="s">
-        <v>892</v>
+        <v>1098</v>
       </c>
       <c r="K106" t="s">
         <v>893</v>
@@ -12731,13 +13284,13 @@
         <v>590</v>
       </c>
       <c r="H107" s="43" t="s">
-        <v>591</v>
+        <v>1099</v>
       </c>
       <c r="I107" s="43" t="s">
         <v>592</v>
       </c>
       <c r="J107" t="s">
-        <v>895</v>
+        <v>1100</v>
       </c>
       <c r="K107" t="s">
         <v>896</v>
@@ -12779,10 +13332,10 @@
         <v>594</v>
       </c>
       <c r="I108" s="43" t="s">
-        <v>595</v>
+        <v>1101</v>
       </c>
       <c r="J108" t="s">
-        <v>898</v>
+        <v>1102</v>
       </c>
       <c r="K108" t="s">
         <v>899</v>
@@ -12827,7 +13380,7 @@
         <v>598</v>
       </c>
       <c r="J109" t="s">
-        <v>901</v>
+        <v>1103</v>
       </c>
       <c r="K109" t="s">
         <v>902</v>
@@ -12872,7 +13425,7 @@
         <v>601</v>
       </c>
       <c r="J110" t="s">
-        <v>904</v>
+        <v>1104</v>
       </c>
       <c r="K110" t="s">
         <v>840</v>
@@ -12911,13 +13464,13 @@
         <v>602</v>
       </c>
       <c r="H111" s="43" t="s">
-        <v>603</v>
+        <v>1105</v>
       </c>
       <c r="I111" s="43" t="s">
         <v>604</v>
       </c>
       <c r="J111" t="s">
-        <v>906</v>
+        <v>1106</v>
       </c>
       <c r="K111" t="s">
         <v>907</v>
@@ -12956,13 +13509,13 @@
         <v>605</v>
       </c>
       <c r="H112" s="43" t="s">
-        <v>606</v>
+        <v>1107</v>
       </c>
       <c r="I112" s="43" t="s">
         <v>607</v>
       </c>
       <c r="J112" t="s">
-        <v>909</v>
+        <v>1108</v>
       </c>
       <c r="K112" t="s">
         <v>910</v>
@@ -13007,7 +13560,7 @@
         <v>608</v>
       </c>
       <c r="J113" t="s">
-        <v>912</v>
+        <v>1109</v>
       </c>
       <c r="K113" t="s">
         <v>913</v>
@@ -13052,7 +13605,7 @@
         <v>614</v>
       </c>
       <c r="J114" s="26" t="s">
-        <v>915</v>
+        <v>1110</v>
       </c>
       <c r="K114" t="s">
         <v>916</v>
@@ -13097,7 +13650,7 @@
         <v>617</v>
       </c>
       <c r="J115" t="s">
-        <v>918</v>
+        <v>1111</v>
       </c>
       <c r="K115" t="s">
         <v>919</v>
@@ -13142,7 +13695,7 @@
         <v>620</v>
       </c>
       <c r="J116" t="s">
-        <v>921</v>
+        <v>1112</v>
       </c>
       <c r="K116" t="s">
         <v>922</v>
@@ -13187,7 +13740,7 @@
         <v>623</v>
       </c>
       <c r="J117" t="s">
-        <v>924</v>
+        <v>1113</v>
       </c>
       <c r="K117" t="s">
         <v>925</v>
@@ -13223,7 +13776,7 @@
         <v>50</v>
       </c>
       <c r="G118" s="46" t="s">
-        <v>624</v>
+        <v>1114</v>
       </c>
       <c r="H118" s="43" t="s">
         <v>625</v>
@@ -13232,7 +13785,7 @@
         <v>626</v>
       </c>
       <c r="J118" t="s">
-        <v>927</v>
+        <v>1115</v>
       </c>
       <c r="K118" t="s">
         <v>928</v>
@@ -13277,7 +13830,7 @@
         <v>629</v>
       </c>
       <c r="J119" t="s">
-        <v>930</v>
+        <v>1116</v>
       </c>
       <c r="K119" t="s">
         <v>931</v>
@@ -13322,7 +13875,7 @@
         <v>632</v>
       </c>
       <c r="J120" t="s">
-        <v>933</v>
+        <v>1117</v>
       </c>
       <c r="K120" t="s">
         <v>934</v>
@@ -13367,7 +13920,7 @@
         <v>635</v>
       </c>
       <c r="J121" t="s">
-        <v>936</v>
+        <v>1118</v>
       </c>
       <c r="K121" t="s">
         <v>937</v>
@@ -13406,13 +13959,13 @@
         <v>636</v>
       </c>
       <c r="H122" s="43" t="s">
-        <v>637</v>
+        <v>1119</v>
       </c>
       <c r="I122" s="43" t="s">
         <v>638</v>
       </c>
       <c r="J122" t="s">
-        <v>939</v>
+        <v>1120</v>
       </c>
       <c r="K122" t="s">
         <v>940</v>
@@ -13451,13 +14004,13 @@
         <v>639</v>
       </c>
       <c r="H123" s="43" t="s">
-        <v>640</v>
+        <v>1121</v>
       </c>
       <c r="I123" s="43" t="s">
         <v>641</v>
       </c>
       <c r="J123" t="s">
-        <v>942</v>
+        <v>1122</v>
       </c>
       <c r="K123" t="s">
         <v>943</v>
@@ -13502,7 +14055,7 @@
         <v>644</v>
       </c>
       <c r="J124" t="s">
-        <v>945</v>
+        <v>1123</v>
       </c>
       <c r="K124" t="s">
         <v>946</v>
@@ -13541,13 +14094,13 @@
         <v>647</v>
       </c>
       <c r="H125" s="43" t="s">
-        <v>648</v>
+        <v>1124</v>
       </c>
       <c r="I125" s="43" t="s">
         <v>649</v>
       </c>
       <c r="J125" s="26" t="s">
-        <v>949</v>
+        <v>1125</v>
       </c>
       <c r="K125" t="s">
         <v>950</v>
@@ -13592,7 +14145,7 @@
         <v>652</v>
       </c>
       <c r="J126" t="s">
-        <v>952</v>
+        <v>1126</v>
       </c>
       <c r="K126" t="s">
         <v>953</v>
@@ -13637,7 +14190,7 @@
         <v>655</v>
       </c>
       <c r="J127" t="s">
-        <v>955</v>
+        <v>1127</v>
       </c>
       <c r="K127" t="s">
         <v>956</v>
@@ -13682,7 +14235,7 @@
         <v>658</v>
       </c>
       <c r="J128" t="s">
-        <v>958</v>
+        <v>1128</v>
       </c>
       <c r="K128" t="s">
         <v>959</v>
@@ -13718,7 +14271,7 @@
         <v>50</v>
       </c>
       <c r="G129" s="46" t="s">
-        <v>659</v>
+        <v>1129</v>
       </c>
       <c r="H129" s="43" t="s">
         <v>660</v>
@@ -13727,7 +14280,7 @@
         <v>661</v>
       </c>
       <c r="J129" t="s">
-        <v>961</v>
+        <v>1130</v>
       </c>
       <c r="K129" t="s">
         <v>962</v>
@@ -13772,7 +14325,7 @@
         <v>664</v>
       </c>
       <c r="J130" t="s">
-        <v>964</v>
+        <v>1131</v>
       </c>
       <c r="K130" t="s">
         <v>965</v>
@@ -13811,13 +14364,13 @@
         <v>665</v>
       </c>
       <c r="H131" s="43" t="s">
-        <v>666</v>
+        <v>1132</v>
       </c>
       <c r="I131" s="43" t="s">
-        <v>667</v>
+        <v>1133</v>
       </c>
       <c r="J131" t="s">
-        <v>967</v>
+        <v>1134</v>
       </c>
       <c r="K131" t="s">
         <v>968</v>
@@ -13862,7 +14415,7 @@
         <v>670</v>
       </c>
       <c r="J132" t="s">
-        <v>970</v>
+        <v>1135</v>
       </c>
       <c r="K132" t="s">
         <v>971</v>
@@ -13907,7 +14460,7 @@
         <v>673</v>
       </c>
       <c r="J133" t="s">
-        <v>973</v>
+        <v>1136</v>
       </c>
       <c r="K133" t="s">
         <v>974</v>
@@ -13952,7 +14505,7 @@
         <v>676</v>
       </c>
       <c r="J134" t="s">
-        <v>976</v>
+        <v>1137</v>
       </c>
       <c r="K134" t="s">
         <v>977</v>
@@ -13997,7 +14550,7 @@
         <v>679</v>
       </c>
       <c r="J135" t="s">
-        <v>979</v>
+        <v>1138</v>
       </c>
       <c r="K135" t="s">
         <v>980</v>

</xml_diff>